<commit_message>
ogni occorrenza ha il suo testimone, l'opera è derivata (T-44, D-055)
appearsInWitness = qp sulle 723 occorrenze di QP; appearsInWork derivata
(propertyChainAxiom appearsInWitness / witnessOf), colonna LiteraryWork_ID
tolta; capitoli parte dell'opera; pseudo-opere tolte. Il pannello del testo
legge il testimone. IQ6 corretta (estratto obbligatorio solo nel testimone
di riferimento: dopo T-41 restituiva 3 righe).
TBox 1.152 -> 1.158, ABox 26.425 -> 27.136, SHACL conforme.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/Chapters.xlsx
+++ b/data/source/xlsx/Chapters.xlsx
@@ -451,7 +451,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>quer_pasticciaccio_adelphi</t>
+          <t>quer_pasticciaccio</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -476,7 +476,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>quer_pasticciaccio_adelphi</t>
+          <t>quer_pasticciaccio</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -501,7 +501,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>quer_pasticciaccio_adelphi</t>
+          <t>quer_pasticciaccio</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -526,7 +526,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>quer_pasticciaccio_adelphi</t>
+          <t>quer_pasticciaccio</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -551,7 +551,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>quer_pasticciaccio_adelphi</t>
+          <t>quer_pasticciaccio</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>quer_pasticciaccio_adelphi</t>
+          <t>quer_pasticciaccio</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>quer_pasticciaccio_adelphi</t>
+          <t>quer_pasticciaccio</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>quer_pasticciaccio_adelphi</t>
+          <t>quer_pasticciaccio</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -651,7 +651,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>quer_pasticciaccio_adelphi</t>
+          <t>quer_pasticciaccio</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -676,7 +676,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>quer_pasticciaccio_adelphi</t>
+          <t>quer_pasticciaccio</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">

</xml_diff>